<commit_message>
valuation correction in lakuri bot devi sumara sadak and autocad scale in x direction or y of editing
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/लाँकुरी बोट देवी सुमारा सडक/valuation लाँकुरी.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/लाँकुरी बोट देवी सुमारा सडक/valuation लाँकुरी.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C23B98A6-1419-4EFF-8146-D2C8A3464906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D324EE4-7309-4D93-9310-2CC9A4190478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,6 @@
     <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
-    <externalReference r:id="rId13"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
@@ -38,22 +37,22 @@
     <definedName name="description_3">[1]Abstract!$B$169</definedName>
     <definedName name="description_310" localSheetId="0">#REF!</definedName>
     <definedName name="description_310" localSheetId="2">#REF!</definedName>
-    <definedName name="description_310" localSheetId="1">[7]Abstract!$B$60</definedName>
+    <definedName name="description_310" localSheetId="1">[4]Abstract!$B$60</definedName>
     <definedName name="description_310">#REF!</definedName>
     <definedName name="description_312" localSheetId="0">#REF!</definedName>
     <definedName name="description_312" localSheetId="2">#REF!</definedName>
-    <definedName name="description_312" localSheetId="1">[8]Abstract!$B$61</definedName>
+    <definedName name="description_312" localSheetId="1">[5]Abstract!$B$61</definedName>
     <definedName name="description_312">#REF!</definedName>
-    <definedName name="description_4">[4]Abstract!$B$170</definedName>
+    <definedName name="description_4">[6]Abstract!$B$170</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
     <definedName name="description_6" localSheetId="0">#REF!</definedName>
     <definedName name="description_6" localSheetId="2">#REF!</definedName>
-    <definedName name="description_6" localSheetId="1">[7]Abstract!$B$172</definedName>
+    <definedName name="description_6" localSheetId="1">[4]Abstract!$B$172</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
     <definedName name="description_781" localSheetId="0">#REF!</definedName>
     <definedName name="description_781" localSheetId="2">#REF!</definedName>
-    <definedName name="description_781" localSheetId="1">[9]Abstract!$B$299</definedName>
+    <definedName name="description_781" localSheetId="1">[7]Abstract!$B$299</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
@@ -604,7 +603,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -712,92 +711,16 @@
     <xf numFmtId="2" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -835,7 +758,82 @@
     <xf numFmtId="1" fontId="8" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1102,138 +1100,6 @@
       <sheetName val="PPMO_BOQ"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1">
-        <row r="170">
-          <cell r="B170" t="str">
-            <v>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications, PCC Grade M 15, Manual Mixing</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="estimate"/>
-      <sheetName val="valuation"/>
-      <sheetName val="WCR"/>
-      <sheetName val="m"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>Project:-तिनघरे बाटो स्तरोन्नति</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>Location:- Shankharapur Municipality 1</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1">
-        <row r="12">
-          <cell r="G12">
-            <v>63.93</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="estimate"/>
-      <sheetName val="WCR"/>
-      <sheetName val="V"/>
-      <sheetName val="M"/>
-      <sheetName val="original estimate"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="13">
-          <cell r="G13">
-            <v>99.9</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2">
-        <row r="16">
-          <cell r="G16">
-            <v>88.199999999999989</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="Datasheet"/>
-      <sheetName val="Abstract"/>
-      <sheetName val="Quantity_Sheet"/>
-      <sheetName val="District_Rate"/>
-      <sheetName val="Equipment_Rate"/>
-      <sheetName val="Summary_of_Rates"/>
-      <sheetName val="rate (roadway)"/>
-      <sheetName val="manhole"/>
-      <sheetName val="bistar"/>
-      <sheetName val="Rate_Analysis"/>
-      <sheetName val="DWC pipe Rate-analysis"/>
-      <sheetName val="Sheet1"/>
-      <sheetName val="Sheet2"/>
-      <sheetName val="Sheet3"/>
-      <sheetName val="Sheet4"/>
-      <sheetName val="Loading_Unloading"/>
-      <sheetName val="Collection"/>
-      <sheetName val="Transportation"/>
-      <sheetName val="References"/>
-      <sheetName val="BOQ"/>
-      <sheetName val="PPMO_BOQ"/>
-    </sheetNames>
-    <sheetDataSet>
       <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1" refreshError="1">
         <row r="60">
@@ -1271,7 +1137,7 @@
 </externalLink>
 </file>
 
-<file path=xl/externalLinks/externalLink8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -1330,7 +1196,66 @@
 </externalLink>
 </file>
 
-<file path=xl/externalLinks/externalLink9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="Datasheet"/>
+      <sheetName val="Abstract"/>
+      <sheetName val="Quantity_Sheet"/>
+      <sheetName val="District_Rate"/>
+      <sheetName val="Equipment_Rate"/>
+      <sheetName val="Summary_of_Rates"/>
+      <sheetName val="rate (roadway)"/>
+      <sheetName val="manhole"/>
+      <sheetName val="bistar"/>
+      <sheetName val="Rate_Analysis"/>
+      <sheetName val="DWC pipe Rate-analysis"/>
+      <sheetName val="Sheet1"/>
+      <sheetName val="Sheet2"/>
+      <sheetName val="Sheet3"/>
+      <sheetName val="Sheet4"/>
+      <sheetName val="Loading_Unloading"/>
+      <sheetName val="Collection"/>
+      <sheetName val="Transportation"/>
+      <sheetName val="References"/>
+      <sheetName val="BOQ"/>
+      <sheetName val="PPMO_BOQ"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="170">
+          <cell r="B170" t="str">
+            <v>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications, PCC Grade M 15, Manual Mixing</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink7.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
@@ -1384,6 +1309,42 @@
       <sheetData sheetId="18" refreshError="1"/>
       <sheetData sheetId="19" refreshError="1"/>
       <sheetData sheetId="20" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink8.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="estimate"/>
+      <sheetName val="valuation"/>
+      <sheetName val="WCR"/>
+      <sheetName val="m"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="6">
+          <cell r="A6" t="str">
+            <v>Project:-तिनघरे बाटो स्तरोन्नति</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7" t="str">
+            <v>Location:- Shankharapur Municipality 1</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1">
+        <row r="12">
+          <cell r="G12">
+            <v>63.93</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1693,113 +1654,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="70"/>
+      <c r="K4" s="70"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="71"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="71"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="66" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
+      <c r="B7" s="74"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="50" t="s">
+      <c r="H7" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
@@ -2477,11 +2438,11 @@
       <c r="B41" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C41" s="47">
+      <c r="C41" s="72">
         <f>J39</f>
         <v>565661.09314466768</v>
       </c>
-      <c r="D41" s="48"/>
+      <c r="D41" s="73"/>
       <c r="E41" s="33">
         <v>100</v>
       </c>
@@ -2496,21 +2457,21 @@
       <c r="B42" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="51">
+      <c r="C42" s="76">
         <v>500000</v>
       </c>
-      <c r="D42" s="52"/>
+      <c r="D42" s="77"/>
       <c r="E42" s="33"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B43" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C43" s="51">
+      <c r="C43" s="76">
         <f>C42-C45-C46</f>
         <v>475000</v>
       </c>
-      <c r="D43" s="52"/>
+      <c r="D43" s="77"/>
       <c r="E43" s="33">
         <f>C43/C41*100</f>
         <v>83.972542173502262</v>
@@ -2520,11 +2481,11 @@
       <c r="B44" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C44" s="53">
+      <c r="C44" s="78">
         <f>C41-C43</f>
         <v>90661.093144667684</v>
       </c>
-      <c r="D44" s="53"/>
+      <c r="D44" s="78"/>
       <c r="E44" s="33">
         <f>100-E43</f>
         <v>16.027457826497738</v>
@@ -2534,11 +2495,11 @@
       <c r="B45" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="C45" s="47">
+      <c r="C45" s="72">
         <f>C42*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D45" s="48"/>
+      <c r="D45" s="73"/>
       <c r="E45" s="33">
         <v>3</v>
       </c>
@@ -2547,17 +2508,24 @@
       <c r="B46" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C46" s="47">
+      <c r="C46" s="72">
         <f>C42*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D46" s="48"/>
+      <c r="D46" s="73"/>
       <c r="E46" s="33">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="A7:F7"/>
@@ -2566,13 +2534,6 @@
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="C44:D44"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2605,203 +2566,203 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="61" t="s">
+      <c r="A1" s="86" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="61"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
     </row>
     <row r="2" spans="1:13" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="87" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="62"/>
-      <c r="C2" s="62"/>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-    </row>
-    <row r="3" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="63" t="s">
+      <c r="B2" s="87"/>
+      <c r="C2" s="87"/>
+      <c r="D2" s="87"/>
+      <c r="E2" s="87"/>
+      <c r="F2" s="87"/>
+      <c r="G2" s="87"/>
+      <c r="H2" s="87"/>
+      <c r="I2" s="87"/>
+      <c r="J2" s="87"/>
+      <c r="K2" s="87"/>
+    </row>
+    <row r="3" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="63"/>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
-      <c r="G3" s="63"/>
-      <c r="H3" s="63"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="63"/>
-    </row>
-    <row r="4" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="63" t="s">
+      <c r="B3" s="88"/>
+      <c r="C3" s="88"/>
+      <c r="D3" s="88"/>
+      <c r="E3" s="88"/>
+      <c r="F3" s="88"/>
+      <c r="G3" s="88"/>
+      <c r="H3" s="88"/>
+      <c r="I3" s="88"/>
+      <c r="J3" s="88"/>
+      <c r="K3" s="88"/>
+    </row>
+    <row r="4" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="63"/>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
-      <c r="G4" s="63"/>
-      <c r="H4" s="63"/>
-      <c r="I4" s="63"/>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63"/>
+      <c r="B4" s="88"/>
+      <c r="C4" s="88"/>
+      <c r="D4" s="88"/>
+      <c r="E4" s="88"/>
+      <c r="F4" s="88"/>
+      <c r="G4" s="88"/>
+      <c r="H4" s="88"/>
+      <c r="I4" s="88"/>
+      <c r="J4" s="88"/>
+      <c r="K4" s="88"/>
     </row>
     <row r="5" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="65" t="s">
+      <c r="A5" s="89" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="65"/>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
-      <c r="E5" s="65"/>
-      <c r="F5" s="65"/>
-      <c r="G5" s="65"/>
-      <c r="H5" s="65"/>
-      <c r="I5" s="65"/>
-      <c r="J5" s="65"/>
-      <c r="K5" s="65"/>
+      <c r="B5" s="89"/>
+      <c r="C5" s="89"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="89"/>
+      <c r="G5" s="89"/>
+      <c r="H5" s="89"/>
+      <c r="I5" s="89"/>
+      <c r="J5" s="89"/>
+      <c r="K5" s="89"/>
     </row>
     <row r="6" spans="1:13" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A6" s="66" t="s">
+      <c r="A6" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="66"/>
-      <c r="C6" s="67">
+      <c r="B6" s="49"/>
+      <c r="C6" s="90">
         <f>F34</f>
         <v>565661.09314466768</v>
       </c>
-      <c r="D6" s="68"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="66" t="s">
+      <c r="D6" s="91"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49" t="s">
         <v>58</v>
       </c>
-      <c r="I6" s="66"/>
-      <c r="J6" s="67">
+      <c r="I6" s="49"/>
+      <c r="J6" s="90">
         <f>I34</f>
-        <v>584751.77340097865</v>
-      </c>
-      <c r="K6" s="68"/>
+        <v>563256.49796061974</v>
+      </c>
+      <c r="K6" s="91"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="70" t="s">
+      <c r="A7" s="51" t="s">
         <v>59</v>
       </c>
-      <c r="B7" s="70"/>
-      <c r="C7" s="70"/>
-      <c r="D7" s="70"/>
-      <c r="F7" s="71"/>
-      <c r="G7" s="71"/>
-      <c r="I7" s="72" t="s">
+      <c r="B7" s="51"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
+      <c r="F7" s="82"/>
+      <c r="G7" s="82"/>
+      <c r="I7" s="83" t="s">
         <v>60</v>
       </c>
-      <c r="J7" s="72"/>
-      <c r="K7" s="72"/>
+      <c r="J7" s="83"/>
+      <c r="K7" s="83"/>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="58"/>
-      <c r="E8" s="58"/>
-      <c r="F8" s="58"/>
-      <c r="I8" s="73" t="s">
+      <c r="B8" s="66"/>
+      <c r="C8" s="66"/>
+      <c r="D8" s="66"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="66"/>
+      <c r="I8" s="84" t="s">
         <v>61</v>
       </c>
-      <c r="J8" s="73"/>
-      <c r="K8" s="73"/>
+      <c r="J8" s="84"/>
+      <c r="K8" s="84"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="74" t="str">
-        <f>[5]estimate!A7</f>
+      <c r="A9" s="85" t="str">
+        <f>[8]estimate!A7</f>
         <v>Location:- Shankharapur Municipality 1</v>
       </c>
-      <c r="B9" s="74"/>
-      <c r="C9" s="74"/>
-      <c r="D9" s="74"/>
-      <c r="E9" s="74"/>
-      <c r="F9" s="74"/>
-      <c r="I9" s="73" t="s">
+      <c r="B9" s="85"/>
+      <c r="C9" s="85"/>
+      <c r="D9" s="85"/>
+      <c r="E9" s="85"/>
+      <c r="F9" s="85"/>
+      <c r="I9" s="84" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="73"/>
-      <c r="K9" s="73"/>
+      <c r="J9" s="84"/>
+      <c r="K9" s="84"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="75" t="s">
+      <c r="A11" s="80" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="75" t="s">
+      <c r="B11" s="80" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="75" t="s">
+      <c r="C11" s="80" t="s">
         <v>12</v>
       </c>
-      <c r="D11" s="76" t="s">
+      <c r="D11" s="81" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76" t="s">
+      <c r="E11" s="81"/>
+      <c r="F11" s="81"/>
+      <c r="G11" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="H11" s="76"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="75" t="s">
+      <c r="H11" s="81"/>
+      <c r="I11" s="81"/>
+      <c r="J11" s="80" t="s">
         <v>65</v>
       </c>
-      <c r="K11" s="77" t="s">
+      <c r="K11" s="79" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="75"/>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="78" t="s">
+      <c r="A12" s="80"/>
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="78" t="s">
+      <c r="E12" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="F12" s="78" t="s">
+      <c r="F12" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="78" t="s">
+      <c r="G12" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="H12" s="78" t="s">
+      <c r="H12" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="I12" s="78" t="s">
+      <c r="I12" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="75"/>
-      <c r="K12" s="77"/>
-    </row>
-    <row r="13" spans="1:13" s="64" customFormat="1" ht="135" x14ac:dyDescent="0.25">
-      <c r="A13" s="79">
+      <c r="J12" s="80"/>
+      <c r="K12" s="79"/>
+    </row>
+    <row r="13" spans="1:13" s="48" customFormat="1" ht="135" x14ac:dyDescent="0.25">
+      <c r="A13" s="53">
         <f>estimate!A9</f>
         <v>1</v>
       </c>
@@ -2809,620 +2770,633 @@
         <f>estimate!B9</f>
         <v>Earthwork Excavation in Cutting, Roadway Excavation in all types of Soil by Mechanical  Means ., Road way Excavation in  all types of soil  as per Drawing and technical specifications  including  removal of stumps and other deleterious  matter, all lifts and lead as per Drawing and instruction of the Engineer.</v>
       </c>
-      <c r="C13" s="80" t="str">
+      <c r="C13" s="54" t="str">
         <f>estimate!H11</f>
         <v>cum</v>
       </c>
-      <c r="D13" s="80">
+      <c r="D13" s="54">
         <f>estimate!G11</f>
         <v>25.601950624809511</v>
       </c>
-      <c r="E13" s="80">
+      <c r="E13" s="54">
         <f>estimate!I11</f>
         <v>62.95</v>
       </c>
-      <c r="F13" s="80">
+      <c r="F13" s="54">
         <f>D13*E13</f>
         <v>1611.6427918317588</v>
       </c>
-      <c r="G13" s="80">
+      <c r="G13" s="54">
         <f>V!G26</f>
-        <v>26.414392159770337</v>
-      </c>
-      <c r="H13" s="80">
+        <v>27.265642159770337</v>
+      </c>
+      <c r="H13" s="54">
         <f>V!I26</f>
         <v>62.95</v>
       </c>
-      <c r="I13" s="80">
+      <c r="I13" s="54">
         <f>G13*H13</f>
-        <v>1662.7859864575428</v>
-      </c>
-      <c r="J13" s="81">
+        <v>1716.3721739575428</v>
+      </c>
+      <c r="J13" s="55">
         <f>I13-F13</f>
-        <v>51.143194625783963</v>
-      </c>
-      <c r="K13" s="82"/>
-      <c r="M13" s="64">
+        <v>104.72938212578401</v>
+      </c>
+      <c r="K13" s="56"/>
+      <c r="M13" s="48">
         <f>1.25*F13</f>
         <v>2014.5534897896985</v>
       </c>
     </row>
-    <row r="14" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="79"/>
-      <c r="B14" s="86" t="str">
+    <row r="14" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="53"/>
+      <c r="B14" s="60" t="str">
         <f>estimate!B12</f>
         <v>-13% VAT for excavator</v>
       </c>
-      <c r="C14" s="80"/>
-      <c r="D14" s="80"/>
-      <c r="E14" s="80"/>
-      <c r="F14" s="80">
+      <c r="C14" s="54"/>
+      <c r="D14" s="54"/>
+      <c r="E14" s="54"/>
+      <c r="F14" s="54">
         <f>estimate!J12</f>
         <v>172.07071014934473</v>
       </c>
-      <c r="G14" s="80"/>
-      <c r="H14" s="80"/>
-      <c r="I14" s="80">
+      <c r="G14" s="54"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="54">
         <f>V!J27</f>
-        <v>177.53112970581645</v>
-      </c>
-      <c r="J14" s="81">
+        <v>183.25238095581648</v>
+      </c>
+      <c r="J14" s="55">
         <f>I14-F14</f>
-        <v>5.4604195564717202</v>
-      </c>
-      <c r="K14" s="82"/>
-      <c r="M14" s="64">
+        <v>11.181670806471743</v>
+      </c>
+      <c r="K14" s="56"/>
+      <c r="M14" s="48">
         <f t="shared" ref="M14" si="0">1.25*F14</f>
         <v>215.0883876866809</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="83"/>
-      <c r="B15" s="84"/>
-      <c r="C15" s="80"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="80"/>
-      <c r="I15" s="80"/>
-      <c r="J15" s="81"/>
-      <c r="K15" s="82"/>
-    </row>
-    <row r="16" spans="1:13" s="64" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="79">
+    <row r="15" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="57"/>
+      <c r="B15" s="58"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
+      <c r="H15" s="54"/>
+      <c r="I15" s="54"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="56"/>
+    </row>
+    <row r="16" spans="1:13" s="48" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="53">
         <f>estimate!A14</f>
         <v>2</v>
       </c>
-      <c r="B16" s="85" t="str">
+      <c r="B16" s="59" t="str">
         <f>estimate!B14</f>
         <v>Providing and laying of hand pack locally available Stone soling with 150 to 200 mm thick stones and packing with smaller stone on prepared surface as per Drawing and Technical Specifications.</v>
       </c>
-      <c r="C16" s="80" t="str">
+      <c r="C16" s="54" t="str">
         <f>estimate!H16</f>
         <v>cum</v>
       </c>
-      <c r="D16" s="80">
+      <c r="D16" s="54">
         <f>estimate!G16</f>
         <v>25.601950624809511</v>
       </c>
-      <c r="E16" s="80">
+      <c r="E16" s="54">
         <f>estimate!I16</f>
         <v>4458.5200000000004</v>
       </c>
-      <c r="F16" s="80">
+      <c r="F16" s="54">
         <f>D16*E16</f>
         <v>114146.80889972571</v>
       </c>
-      <c r="G16" s="80">
+      <c r="G16" s="54">
         <f>V!G46</f>
-        <v>26.414392159770337</v>
-      </c>
-      <c r="H16" s="80">
+        <v>19.640222480358585</v>
+      </c>
+      <c r="H16" s="54">
         <f>V!I46</f>
         <v>4458.5200000000004</v>
       </c>
-      <c r="I16" s="80">
+      <c r="I16" s="54">
         <f>G16*H16</f>
-        <v>117769.09573217925</v>
-      </c>
-      <c r="J16" s="81">
+        <v>87566.324733128364</v>
+      </c>
+      <c r="J16" s="55">
         <f>I16-F16</f>
-        <v>3622.2868324535375</v>
-      </c>
-      <c r="K16" s="82"/>
-      <c r="M16" s="64">
+        <v>-26580.484166597351</v>
+      </c>
+      <c r="K16" s="56"/>
+      <c r="M16" s="48">
         <f t="shared" ref="M16:M30" si="1">1.25*F16</f>
         <v>142683.51112465715</v>
       </c>
     </row>
-    <row r="17" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="79"/>
-      <c r="B17" s="86" t="str">
+    <row r="17" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="53"/>
+      <c r="B17" s="60" t="str">
         <f>estimate!B17</f>
         <v>-13% VAT for block stone</v>
       </c>
-      <c r="C17" s="80"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="80"/>
-      <c r="F17" s="80">
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
+      <c r="E17" s="54"/>
+      <c r="F17" s="54">
         <f>estimate!J17</f>
         <v>9863.3460530326138</v>
       </c>
-      <c r="G17" s="80"/>
-      <c r="H17" s="80"/>
-      <c r="I17" s="80">
+      <c r="G17" s="54"/>
+      <c r="H17" s="54"/>
+      <c r="I17" s="54">
         <f>V!J47</f>
-        <v>10176.345328931937</v>
-      </c>
-      <c r="J17" s="81">
+        <v>7566.544976248997</v>
+      </c>
+      <c r="J17" s="55">
         <f>I17-F17</f>
-        <v>312.99927589932304</v>
-      </c>
-      <c r="K17" s="82"/>
-      <c r="M17" s="64">
+        <v>-2296.8010767836167</v>
+      </c>
+      <c r="K17" s="56"/>
+      <c r="M17" s="48">
         <f t="shared" ref="M17" si="2">1.25*F17</f>
         <v>12329.182566290767</v>
       </c>
     </row>
-    <row r="18" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="79"/>
-      <c r="B18" s="85"/>
-      <c r="C18" s="80"/>
-      <c r="D18" s="80"/>
-      <c r="E18" s="80"/>
-      <c r="F18" s="80"/>
-      <c r="G18" s="80"/>
-      <c r="H18" s="80"/>
-      <c r="I18" s="80"/>
-      <c r="J18" s="81"/>
-      <c r="K18" s="82"/>
-    </row>
-    <row r="19" spans="1:13" s="64" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="79">
+    <row r="18" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="53"/>
+      <c r="B18" s="59"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="54"/>
+      <c r="E18" s="54"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="55"/>
+      <c r="K18" s="56"/>
+    </row>
+    <row r="19" spans="1:13" s="48" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="53">
         <f>estimate!A19</f>
         <v>3</v>
       </c>
-      <c r="B19" s="85" t="str">
+      <c r="B19" s="59" t="str">
         <f>estimate!B19</f>
         <v>Providing and laying of Plain/Reinforced Cement Concrete in Foundation complete as per Drawing and Technical Specifications., RCC Grade M 20</v>
       </c>
-      <c r="C19" s="80" t="str">
+      <c r="C19" s="54" t="str">
         <f>estimate!H21</f>
         <v>cum</v>
       </c>
-      <c r="D19" s="80">
+      <c r="D19" s="54">
         <f>estimate!G21</f>
         <v>25.601950624809511</v>
       </c>
-      <c r="E19" s="80">
+      <c r="E19" s="54">
         <f>estimate!I21</f>
         <v>12000.5</v>
       </c>
-      <c r="F19" s="80">
+      <c r="F19" s="54">
         <f>D19*E19</f>
         <v>307236.20847302652</v>
       </c>
-      <c r="G19" s="80">
+      <c r="G19" s="54">
         <f>V!G66</f>
-        <v>26.414392159770337</v>
-      </c>
-      <c r="H19" s="80">
+        <v>27.265642159770337</v>
+      </c>
+      <c r="H19" s="54">
         <f>V!I66</f>
         <v>12000.5</v>
       </c>
-      <c r="I19" s="80">
+      <c r="I19" s="54">
         <f>G19*H19</f>
-        <v>316985.91311332391</v>
-      </c>
-      <c r="J19" s="81">
+        <v>327201.33873832395</v>
+      </c>
+      <c r="J19" s="55">
         <f>I19-F19</f>
-        <v>9749.7046402973938</v>
-      </c>
-      <c r="K19" s="82"/>
-      <c r="M19" s="64">
+        <v>19965.130265297426</v>
+      </c>
+      <c r="K19" s="56"/>
+      <c r="M19" s="48">
         <f t="shared" si="1"/>
         <v>384045.26059128315</v>
       </c>
     </row>
-    <row r="20" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="79"/>
-      <c r="B20" s="86" t="str">
+    <row r="20" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="53"/>
+      <c r="B20" s="60" t="str">
         <f>estimate!B22</f>
         <v>-13% VAT for cement</v>
       </c>
-      <c r="C20" s="80"/>
-      <c r="D20" s="80"/>
-      <c r="E20" s="80"/>
-      <c r="F20" s="80">
+      <c r="C20" s="54"/>
+      <c r="D20" s="54"/>
+      <c r="E20" s="54"/>
+      <c r="F20" s="54">
         <f>estimate!J22</f>
         <v>15064.010752819264</v>
       </c>
-      <c r="G20" s="80"/>
-      <c r="H20" s="80"/>
-      <c r="I20" s="80">
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54">
         <f>V!J67</f>
-        <v>15542.045735311067</v>
-      </c>
-      <c r="J20" s="81">
+        <v>16042.915350336069</v>
+      </c>
+      <c r="J20" s="55">
         <f>I20-F20</f>
-        <v>478.03498249180302</v>
-      </c>
-      <c r="K20" s="82"/>
-      <c r="M20" s="64">
+        <v>978.90459751680464</v>
+      </c>
+      <c r="K20" s="56"/>
+      <c r="M20" s="48">
         <f t="shared" si="1"/>
         <v>18830.013441024079</v>
       </c>
     </row>
-    <row r="21" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="79"/>
-      <c r="B21" s="86" t="str">
+    <row r="21" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="53"/>
+      <c r="B21" s="60" t="str">
         <f>estimate!B23</f>
         <v>-13% VAT for sand</v>
       </c>
-      <c r="C21" s="80"/>
-      <c r="D21" s="80"/>
-      <c r="E21" s="80"/>
-      <c r="F21" s="80">
+      <c r="C21" s="54"/>
+      <c r="D21" s="54"/>
+      <c r="E21" s="54"/>
+      <c r="F21" s="54">
         <f>estimate!J23</f>
         <v>4755.5418469978658</v>
       </c>
-      <c r="G21" s="80"/>
-      <c r="H21" s="80"/>
-      <c r="I21" s="80">
+      <c r="G21" s="54"/>
+      <c r="H21" s="54"/>
+      <c r="I21" s="54">
         <f>V!J68</f>
-        <v>4906.4522121636119</v>
-      </c>
-      <c r="J21" s="81">
+        <v>5064.5712186636119</v>
+      </c>
+      <c r="J21" s="55">
         <f t="shared" ref="J21:J24" si="3">I21-F21</f>
-        <v>150.91036516574604</v>
-      </c>
-      <c r="K21" s="82"/>
-    </row>
-    <row r="22" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="79"/>
-      <c r="B22" s="86" t="str">
+        <v>309.02937166574611</v>
+      </c>
+      <c r="K21" s="56"/>
+    </row>
+    <row r="22" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="53"/>
+      <c r="B22" s="60" t="str">
         <f>estimate!B24</f>
         <v>-13% VAT for aggregate</v>
       </c>
-      <c r="C22" s="80"/>
-      <c r="D22" s="80"/>
-      <c r="E22" s="80"/>
-      <c r="F22" s="80">
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
+      <c r="E22" s="54"/>
+      <c r="F22" s="54">
         <f>estimate!J24</f>
         <v>9828.1198171289252</v>
       </c>
-      <c r="G22" s="80"/>
-      <c r="H22" s="80"/>
-      <c r="I22" s="80">
+      <c r="G22" s="54"/>
+      <c r="H22" s="54"/>
+      <c r="I22" s="54">
         <f>V!J69</f>
-        <v>10140.001238471466</v>
-      </c>
-      <c r="J22" s="81">
+        <v>10466.780518571466</v>
+      </c>
+      <c r="J22" s="55">
         <f t="shared" si="3"/>
-        <v>311.88142134254122</v>
-      </c>
-      <c r="K22" s="82"/>
-    </row>
-    <row r="23" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="79"/>
-      <c r="B23" s="86" t="str">
+        <v>638.66070144254081</v>
+      </c>
+      <c r="K22" s="56"/>
+    </row>
+    <row r="23" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="53"/>
+      <c r="B23" s="60" t="str">
         <f>estimate!B25</f>
         <v>-13% VAT for water</v>
       </c>
-      <c r="C23" s="80"/>
-      <c r="D23" s="80"/>
-      <c r="E23" s="80"/>
-      <c r="F23" s="80">
+      <c r="C23" s="54"/>
+      <c r="D23" s="54"/>
+      <c r="E23" s="54"/>
+      <c r="F23" s="54">
         <f>estimate!J25</f>
         <v>171.95976836330388</v>
       </c>
-      <c r="G23" s="80"/>
-      <c r="H23" s="80"/>
-      <c r="I23" s="80">
+      <c r="G23" s="54"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54">
         <f>V!J70</f>
-        <v>177.41666733979076</v>
-      </c>
-      <c r="J23" s="81">
+        <v>183.13422983979078</v>
+      </c>
+      <c r="J23" s="55">
         <f t="shared" si="3"/>
-        <v>5.4568989764868832</v>
-      </c>
-      <c r="K23" s="82"/>
-    </row>
-    <row r="24" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="79"/>
-      <c r="B24" s="86" t="str">
+        <v>11.174461476486897</v>
+      </c>
+      <c r="K23" s="56"/>
+    </row>
+    <row r="24" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="53"/>
+      <c r="B24" s="60" t="str">
         <f>estimate!B26</f>
         <v>-13% VAT for formwork</v>
       </c>
-      <c r="C24" s="80"/>
-      <c r="D24" s="80"/>
-      <c r="E24" s="80"/>
-      <c r="F24" s="80">
+      <c r="C24" s="54"/>
+      <c r="D24" s="54"/>
+      <c r="E24" s="54"/>
+      <c r="F24" s="54">
         <f>estimate!J26</f>
         <v>1536.18872295032</v>
       </c>
-      <c r="G24" s="80"/>
-      <c r="H24" s="80"/>
-      <c r="I24" s="80">
+      <c r="G24" s="54"/>
+      <c r="H24" s="54"/>
+      <c r="I24" s="54">
         <f>V!J71</f>
-        <v>1584.9374898842677</v>
-      </c>
-      <c r="J24" s="81">
+        <v>1636.0148733842677</v>
+      </c>
+      <c r="J24" s="55">
         <f t="shared" si="3"/>
-        <v>48.748766933947763</v>
-      </c>
-      <c r="K24" s="82"/>
-    </row>
-    <row r="25" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="83"/>
-      <c r="B25" s="84"/>
-      <c r="C25" s="80"/>
-      <c r="D25" s="80"/>
-      <c r="E25" s="80"/>
-      <c r="F25" s="80"/>
-      <c r="G25" s="80"/>
-      <c r="H25" s="80"/>
-      <c r="I25" s="80"/>
-      <c r="J25" s="81"/>
-      <c r="K25" s="82"/>
-    </row>
-    <row r="26" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="79">
+        <v>99.82615043394776</v>
+      </c>
+      <c r="K24" s="56"/>
+    </row>
+    <row r="25" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="57"/>
+      <c r="B25" s="58"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="54"/>
+      <c r="E25" s="54"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="54"/>
+      <c r="I25" s="54"/>
+      <c r="J25" s="55"/>
+      <c r="K25" s="56"/>
+    </row>
+    <row r="26" spans="1:13" s="48" customFormat="1" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="53">
         <f>estimate!A28</f>
         <v>4</v>
       </c>
-      <c r="B26" s="85" t="str">
+      <c r="B26" s="59" t="str">
         <f>estimate!B28</f>
         <v xml:space="preserve">Providing and laying , fitting and placing HYSD bar reinforcement in sub-structure complete as per Drawing and Technical Specifications and instruction of site engineer  </v>
       </c>
-      <c r="C26" s="80" t="str">
+      <c r="C26" s="54" t="str">
         <f>estimate!H31</f>
         <v>tonne</v>
       </c>
-      <c r="D26" s="80">
+      <c r="D26" s="54">
         <f>estimate!G31</f>
         <v>0.69012345679012344</v>
       </c>
-      <c r="E26" s="80">
+      <c r="E26" s="54">
         <f>estimate!I31</f>
         <v>124355</v>
       </c>
-      <c r="F26" s="80">
+      <c r="F26" s="54">
         <f>D26*E26</f>
         <v>85820.3024691358</v>
       </c>
-      <c r="G26" s="80">
+      <c r="G26" s="54">
         <f>V!G102</f>
         <v>0.7214972839506173</v>
       </c>
-      <c r="H26" s="80">
+      <c r="H26" s="54">
         <f>V!I102</f>
         <v>124355</v>
       </c>
-      <c r="I26" s="80">
+      <c r="I26" s="54">
         <f>G26*H26</f>
         <v>89721.794745679013</v>
       </c>
-      <c r="J26" s="81">
+      <c r="J26" s="55">
         <f>I26-F26</f>
         <v>3901.4922765432129</v>
       </c>
-      <c r="K26" s="82"/>
-      <c r="M26" s="64">
+      <c r="K26" s="56"/>
+      <c r="M26" s="48">
         <f t="shared" si="1"/>
         <v>107275.37808641975</v>
       </c>
     </row>
-    <row r="27" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="79"/>
-      <c r="B27" s="86" t="str">
+    <row r="27" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="53"/>
+      <c r="B27" s="60" t="str">
         <f>estimate!B32</f>
         <v>-13% VAT for HYSD bar</v>
       </c>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="80"/>
-      <c r="F27" s="80">
+      <c r="C27" s="54"/>
+      <c r="D27" s="54"/>
+      <c r="E27" s="54"/>
+      <c r="F27" s="54">
         <f>estimate!J32</f>
         <v>9868.7654320987658</v>
       </c>
-      <c r="G27" s="80"/>
-      <c r="H27" s="80"/>
-      <c r="I27" s="80">
+      <c r="G27" s="54"/>
+      <c r="H27" s="54"/>
+      <c r="I27" s="54">
         <f>V!J103</f>
         <v>10317.411160493828</v>
       </c>
-      <c r="J27" s="81">
+      <c r="J27" s="55">
         <f>I27-F27</f>
         <v>448.64572839506218</v>
       </c>
-      <c r="K27" s="82"/>
-      <c r="M27" s="64">
+      <c r="K27" s="56"/>
+      <c r="M27" s="48">
         <f t="shared" si="1"/>
         <v>12335.956790123457</v>
       </c>
     </row>
-    <row r="28" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="79"/>
-      <c r="B28" s="86" t="str">
+    <row r="28" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="53"/>
+      <c r="B28" s="60" t="str">
         <f>estimate!B33</f>
         <v>-13% VAT for binding wire</v>
       </c>
-      <c r="C28" s="80"/>
-      <c r="D28" s="80"/>
-      <c r="E28" s="80"/>
-      <c r="F28" s="80">
+      <c r="C28" s="54"/>
+      <c r="D28" s="54"/>
+      <c r="E28" s="54"/>
+      <c r="F28" s="54">
         <f>estimate!J33</f>
         <v>86.127407407407404</v>
       </c>
-      <c r="G28" s="80"/>
-      <c r="H28" s="80"/>
-      <c r="I28" s="80">
+      <c r="G28" s="54"/>
+      <c r="H28" s="54"/>
+      <c r="I28" s="54">
         <f>V!J104</f>
         <v>90.042861037037042</v>
       </c>
-      <c r="J28" s="81">
+      <c r="J28" s="55">
         <f>I28-F28</f>
         <v>3.9154536296296385</v>
       </c>
-      <c r="K28" s="82"/>
-    </row>
-    <row r="29" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="83"/>
-      <c r="B29" s="84"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="80"/>
-      <c r="F29" s="80"/>
-      <c r="G29" s="80"/>
-      <c r="H29" s="80"/>
-      <c r="I29" s="80"/>
-      <c r="J29" s="81"/>
-      <c r="K29" s="82"/>
-    </row>
-    <row r="30" spans="1:13" s="64" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="79">
+      <c r="K28" s="56"/>
+    </row>
+    <row r="29" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="57"/>
+      <c r="B29" s="58"/>
+      <c r="C29" s="54"/>
+      <c r="D29" s="54"/>
+      <c r="E29" s="54"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="54"/>
+      <c r="I29" s="54"/>
+      <c r="J29" s="55"/>
+      <c r="K29" s="56"/>
+    </row>
+    <row r="30" spans="1:13" s="48" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="53">
         <f>estimate!A35</f>
         <v>5</v>
       </c>
-      <c r="B30" s="91" t="str">
+      <c r="B30" s="65" t="str">
         <f>estimate!B35</f>
         <v>Provisional sum for lab tests</v>
       </c>
-      <c r="C30" s="80" t="str">
+      <c r="C30" s="54" t="str">
         <f>estimate!H35</f>
         <v>PS</v>
       </c>
-      <c r="D30" s="80">
+      <c r="D30" s="54">
         <f>estimate!G35</f>
         <v>1</v>
       </c>
-      <c r="E30" s="80">
+      <c r="E30" s="54">
         <f>estimate!I35</f>
         <v>5000</v>
       </c>
-      <c r="F30" s="80">
+      <c r="F30" s="54">
         <f>D30*E30</f>
         <v>5000</v>
       </c>
-      <c r="G30" s="80">
+      <c r="G30" s="54">
         <f>V!G106</f>
         <v>1</v>
       </c>
-      <c r="H30" s="80">
+      <c r="H30" s="54">
         <f>V!I106</f>
         <v>5000</v>
       </c>
-      <c r="I30" s="80">
+      <c r="I30" s="54">
         <f>G30*H30</f>
         <v>5000</v>
       </c>
-      <c r="J30" s="81">
+      <c r="J30" s="55">
         <f>I30-F30</f>
         <v>0</v>
       </c>
-      <c r="K30" s="82"/>
-      <c r="M30" s="64">
+      <c r="K30" s="56"/>
+      <c r="M30" s="48">
         <f t="shared" si="1"/>
         <v>6250</v>
       </c>
     </row>
-    <row r="31" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="83"/>
-      <c r="B31" s="84"/>
-      <c r="C31" s="80"/>
-      <c r="D31" s="80"/>
-      <c r="E31" s="80"/>
-      <c r="F31" s="80"/>
-      <c r="G31" s="80"/>
-      <c r="H31" s="80"/>
-      <c r="I31" s="80"/>
-      <c r="J31" s="81"/>
-      <c r="K31" s="82"/>
-    </row>
-    <row r="32" spans="1:13" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="79">
+    <row r="31" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="57"/>
+      <c r="B31" s="58"/>
+      <c r="C31" s="54"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="54"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="54"/>
+      <c r="I31" s="54"/>
+      <c r="J31" s="55"/>
+      <c r="K31" s="56"/>
+    </row>
+    <row r="32" spans="1:13" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="53">
         <f>estimate!A37</f>
         <v>6</v>
       </c>
-      <c r="B32" s="87" t="str">
+      <c r="B32" s="61" t="str">
         <f>estimate!B37</f>
         <v>Information board (सुचना पाटि)</v>
       </c>
-      <c r="C32" s="80" t="str">
+      <c r="C32" s="54" t="str">
         <f>estimate!H37</f>
         <v>no.</v>
       </c>
-      <c r="D32" s="80">
+      <c r="D32" s="54">
         <f>estimate!G37</f>
         <v>1</v>
       </c>
-      <c r="E32" s="80">
+      <c r="E32" s="54">
         <f>estimate!I37</f>
         <v>500</v>
       </c>
-      <c r="F32" s="80">
+      <c r="F32" s="54">
         <f>D32*E32</f>
         <v>500</v>
       </c>
-      <c r="G32" s="80">
+      <c r="G32" s="54">
         <f>V!G108</f>
         <v>1</v>
       </c>
-      <c r="H32" s="80">
+      <c r="H32" s="54">
         <f>V!I108</f>
         <v>500</v>
       </c>
-      <c r="I32" s="80">
+      <c r="I32" s="54">
         <f>G32*H32</f>
         <v>500</v>
       </c>
-      <c r="J32" s="81">
+      <c r="J32" s="55">
         <f>I32-F32</f>
         <v>0</v>
       </c>
-      <c r="K32" s="82"/>
-    </row>
-    <row r="33" spans="1:11" s="64" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="84"/>
-      <c r="B33" s="84"/>
-      <c r="C33" s="80"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="80"/>
-      <c r="F33" s="80"/>
-      <c r="G33" s="80"/>
-      <c r="H33" s="80"/>
-      <c r="I33" s="80"/>
-      <c r="J33" s="81"/>
-      <c r="K33" s="82"/>
+      <c r="K32" s="56"/>
+    </row>
+    <row r="33" spans="1:11" s="48" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="58"/>
+      <c r="B33" s="58"/>
+      <c r="C33" s="54"/>
+      <c r="D33" s="54"/>
+      <c r="E33" s="54"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="54"/>
+      <c r="H33" s="54"/>
+      <c r="I33" s="54"/>
+      <c r="J33" s="55"/>
+      <c r="K33" s="56"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="41"/>
-      <c r="B34" s="88" t="s">
+      <c r="B34" s="62" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="88"/>
-      <c r="D34" s="89"/>
-      <c r="E34" s="89"/>
-      <c r="F34" s="89">
+      <c r="C34" s="62"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63">
         <f>SUM(F13:F32)</f>
         <v>565661.09314466768</v>
       </c>
-      <c r="G34" s="89"/>
-      <c r="H34" s="89"/>
-      <c r="I34" s="89">
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63">
         <f>SUM(I13:I32)</f>
-        <v>584751.77340097865</v>
-      </c>
-      <c r="J34" s="90">
+        <v>563256.49796061974</v>
+      </c>
+      <c r="J34" s="64">
         <f>I34-F34</f>
-        <v>19090.680256310967</v>
+        <v>-2404.5951840479393</v>
       </c>
       <c r="K34" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="I9:K9"/>
     <mergeCell ref="K11:K12"/>
     <mergeCell ref="A11:A12"/>
     <mergeCell ref="B11:B12"/>
@@ -3430,19 +3404,6 @@
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="G11:I11"/>
     <mergeCell ref="J11:J12"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="J6:K6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3475,113 +3436,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
     </row>
     <row r="2" spans="1:11" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="56"/>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="56"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="56"/>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="70"/>
+      <c r="K4" s="70"/>
     </row>
     <row r="5" spans="1:11" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="71" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="57"/>
-      <c r="C5" s="57"/>
-      <c r="D5" s="57"/>
-      <c r="E5" s="57"/>
-      <c r="F5" s="57"/>
-      <c r="G5" s="57"/>
-      <c r="H5" s="57"/>
-      <c r="I5" s="57"/>
-      <c r="J5" s="57"/>
-      <c r="K5" s="57"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
+      <c r="E5" s="71"/>
+      <c r="F5" s="71"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
+      <c r="J5" s="71"/>
+      <c r="K5" s="71"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="66" t="s">
         <v>49</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="58"/>
+      <c r="B6" s="66"/>
+      <c r="C6" s="66"/>
+      <c r="D6" s="66"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="66"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="59" t="s">
+      <c r="H6" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="I6" s="59"/>
-      <c r="J6" s="59"/>
-      <c r="K6" s="59"/>
+      <c r="I6" s="67"/>
+      <c r="J6" s="67"/>
+      <c r="K6" s="67"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
+      <c r="B7" s="74"/>
+      <c r="C7" s="74"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="74"/>
       <c r="G7" s="5"/>
-      <c r="H7" s="50" t="s">
+      <c r="H7" s="75" t="s">
         <v>68</v>
       </c>
-      <c r="I7" s="50"/>
-      <c r="J7" s="50"/>
-      <c r="K7" s="50"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="75"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
@@ -4043,7 +4004,7 @@
       <c r="A25" s="10"/>
       <c r="B25" s="16"/>
       <c r="C25" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="14">
         <f>'chainage measurement'!C18</f>
@@ -4058,7 +4019,7 @@
       </c>
       <c r="G25" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.85125000000000006</v>
       </c>
       <c r="H25" s="12"/>
       <c r="I25" s="12"/>
@@ -4076,7 +4037,7 @@
       <c r="F26" s="18"/>
       <c r="G26" s="19">
         <f>SUM(G10:G25)</f>
-        <v>26.414392159770337</v>
+        <v>27.265642159770337</v>
       </c>
       <c r="H26" s="20" t="s">
         <v>27</v>
@@ -4086,7 +4047,7 @@
       </c>
       <c r="J26" s="19">
         <f>G26*I26</f>
-        <v>1662.7859864575428</v>
+        <v>1716.3721739575428</v>
       </c>
       <c r="K26" s="18"/>
     </row>
@@ -4104,7 +4065,7 @@
       <c r="I27" s="12"/>
       <c r="J27" s="13">
         <f>0.13*G26*18612/360</f>
-        <v>177.53112970581645</v>
+        <v>183.25238095581648</v>
       </c>
       <c r="K27" s="12"/>
     </row>
@@ -4173,19 +4134,19 @@
       <c r="A31" s="10"/>
       <c r="B31" s="16"/>
       <c r="C31" s="12">
-        <f>C11</f>
+        <f t="shared" ref="C31:F45" si="2">C11</f>
         <v>1</v>
       </c>
       <c r="D31" s="14">
-        <f>D11</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E31" s="14">
-        <f>E11</f>
+        <f t="shared" si="2"/>
         <v>3.3145382505333738</v>
       </c>
       <c r="F31" s="14">
-        <f>F11</f>
+        <f t="shared" si="2"/>
         <v>0.12699380270242813</v>
       </c>
       <c r="G31" s="14">
@@ -4201,19 +4162,19 @@
       <c r="A32" s="10"/>
       <c r="B32" s="16"/>
       <c r="C32" s="12">
-        <f>C12</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D32" s="14">
-        <f>D12</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E32" s="14">
-        <f>E12</f>
+        <f t="shared" si="2"/>
         <v>3.0219445291069795</v>
       </c>
       <c r="F32" s="14">
-        <f>F12</f>
+        <f t="shared" si="2"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G32" s="14">
@@ -4229,19 +4190,19 @@
       <c r="A33" s="10"/>
       <c r="B33" s="16"/>
       <c r="C33" s="12">
-        <f>C13</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D33" s="14">
-        <f>D13</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E33" s="14">
-        <f>E13</f>
+        <f t="shared" si="2"/>
         <v>2.9838463882962509</v>
       </c>
       <c r="F33" s="14">
-        <f>F13</f>
+        <f t="shared" si="2"/>
         <v>0.11033729553997765</v>
       </c>
       <c r="G33" s="14">
@@ -4257,19 +4218,19 @@
       <c r="A34" s="10"/>
       <c r="B34" s="16"/>
       <c r="C34" s="12">
-        <f>C14</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D34" s="14">
-        <f>D14</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E34" s="14">
-        <f>E14</f>
+        <f t="shared" si="2"/>
         <v>3.1621456872904599</v>
       </c>
       <c r="F34" s="14">
-        <f>F14</f>
+        <f t="shared" si="2"/>
         <v>0.11668698567509903</v>
       </c>
       <c r="G34" s="14">
@@ -4285,19 +4246,19 @@
       <c r="A35" s="10"/>
       <c r="B35" s="16"/>
       <c r="C35" s="12">
-        <f>C15</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D35" s="14">
-        <f>D15</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E35" s="14">
-        <f>E15</f>
+        <f t="shared" si="2"/>
         <v>3.0859494056690031</v>
       </c>
       <c r="F35" s="14">
-        <f>F15</f>
+        <f t="shared" si="2"/>
         <v>0.11668698567509903</v>
       </c>
       <c r="G35" s="14">
@@ -4313,19 +4274,19 @@
       <c r="A36" s="10"/>
       <c r="B36" s="16"/>
       <c r="C36" s="12">
-        <f>C16</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D36" s="14">
-        <f>D16</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E36" s="14">
-        <f>E16</f>
+        <f t="shared" si="2"/>
         <v>3.1366961292288935</v>
       </c>
       <c r="F36" s="14">
-        <f>F16</f>
+        <f t="shared" si="2"/>
         <v>0.11033729553997765</v>
       </c>
       <c r="G36" s="14">
@@ -4341,19 +4302,19 @@
       <c r="A37" s="10"/>
       <c r="B37" s="16"/>
       <c r="C37" s="12">
-        <f>C17</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D37" s="14">
-        <f>D17</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E37" s="14">
-        <f>E17</f>
+        <f t="shared" si="2"/>
         <v>3.1366961292288935</v>
       </c>
       <c r="F37" s="14">
-        <f>F17</f>
+        <f t="shared" si="2"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G37" s="14">
@@ -4369,19 +4330,19 @@
       <c r="A38" s="10"/>
       <c r="B38" s="16"/>
       <c r="C38" s="12">
-        <f>C18</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D38" s="14">
-        <f>D18</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E38" s="14">
-        <f>E18</f>
+        <f t="shared" si="2"/>
         <v>3.1240475464797317</v>
       </c>
       <c r="F38" s="14">
-        <f>F18</f>
+        <f t="shared" si="2"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G38" s="14">
@@ -4397,19 +4358,19 @@
       <c r="A39" s="10"/>
       <c r="B39" s="16"/>
       <c r="C39" s="12">
-        <f>C19</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D39" s="14">
-        <f>D19</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E39" s="14">
-        <f>E19</f>
+        <f t="shared" si="2"/>
         <v>3.2002438281011885</v>
       </c>
       <c r="F39" s="14">
-        <f>F19</f>
+        <f t="shared" si="2"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G39" s="14">
@@ -4425,19 +4386,19 @@
       <c r="A40" s="10"/>
       <c r="B40" s="16"/>
       <c r="C40" s="12">
-        <f>C20</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D40" s="14">
-        <f>D20</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E40" s="14">
-        <f>E20</f>
+        <f t="shared" si="2"/>
         <v>3.1240475464797317</v>
       </c>
       <c r="F40" s="14">
-        <f>F20</f>
+        <f t="shared" si="2"/>
         <v>7.8588844864370622E-2</v>
       </c>
       <c r="G40" s="14">
@@ -4453,19 +4414,19 @@
       <c r="A41" s="10"/>
       <c r="B41" s="16"/>
       <c r="C41" s="12">
-        <f>C21</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="D41" s="14">
-        <f>D21</f>
+        <f t="shared" si="2"/>
         <v>3.047851264858275</v>
       </c>
       <c r="E41" s="14">
-        <f>E21</f>
+        <f t="shared" si="2"/>
         <v>3.2002438281011885</v>
       </c>
       <c r="F41" s="14">
-        <f>F21</f>
+        <f t="shared" si="2"/>
         <v>6.5889464594127783E-2</v>
       </c>
       <c r="G41" s="14">
@@ -4481,24 +4442,23 @@
       <c r="A42" s="10"/>
       <c r="B42" s="16"/>
       <c r="C42" s="12">
-        <f>C22</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D42" s="14">
-        <f>D22</f>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
       <c r="E42" s="14">
-        <f>E22</f>
+        <f t="shared" si="2"/>
         <v>3.5557756781469063</v>
       </c>
       <c r="F42" s="14">
-        <f>F22</f>
+        <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
       <c r="G42" s="14">
         <f t="shared" si="1"/>
-        <v>3.2001981103322157</v>
+        <v>0</v>
       </c>
       <c r="H42" s="12"/>
       <c r="I42" s="12"/>
@@ -4509,24 +4469,23 @@
       <c r="A43" s="10"/>
       <c r="B43" s="16"/>
       <c r="C43" s="12">
-        <f>C23</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="14">
-        <f>D23</f>
+        <f t="shared" si="2"/>
         <v>0.35558264756679875</v>
       </c>
       <c r="E43" s="14">
-        <f>E23</f>
+        <f t="shared" si="2"/>
         <v>3.8351112465711674</v>
       </c>
       <c r="F43" s="14">
-        <f>F23</f>
+        <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
       <c r="G43" s="14">
         <f t="shared" si="1"/>
-        <v>0.20455485161534726</v>
+        <v>0</v>
       </c>
       <c r="H43" s="12"/>
       <c r="I43" s="12"/>
@@ -4537,24 +4496,23 @@
       <c r="A44" s="10"/>
       <c r="B44" s="16"/>
       <c r="C44" s="12">
-        <f>C24</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D44" s="14">
-        <f>D24</f>
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
       <c r="E44" s="14">
-        <f>E24</f>
+        <f t="shared" si="2"/>
         <v>4.4925556232855843</v>
       </c>
       <c r="F44" s="14">
-        <f>F24</f>
+        <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
       <c r="G44" s="14">
         <f t="shared" si="1"/>
-        <v>3.3694167174641878</v>
+        <v>0</v>
       </c>
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
@@ -4565,19 +4523,18 @@
       <c r="A45" s="10"/>
       <c r="B45" s="16"/>
       <c r="C45" s="12">
-        <f>C25</f>
         <v>0</v>
       </c>
       <c r="D45" s="14">
-        <f>D25</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="E45" s="14">
-        <f>E25</f>
+        <f t="shared" si="2"/>
         <v>5.6750000000000007</v>
       </c>
       <c r="F45" s="14">
-        <f>F25</f>
+        <f t="shared" si="2"/>
         <v>0.15</v>
       </c>
       <c r="G45" s="14">
@@ -4600,7 +4557,7 @@
       <c r="F46" s="18"/>
       <c r="G46" s="19">
         <f>SUM(G30:G45)</f>
-        <v>26.414392159770337</v>
+        <v>19.640222480358585</v>
       </c>
       <c r="H46" s="20" t="s">
         <v>27</v>
@@ -4610,7 +4567,7 @@
       </c>
       <c r="J46" s="19">
         <f>G46*I46</f>
-        <v>117769.09573217925</v>
+        <v>87566.324733128364</v>
       </c>
       <c r="K46" s="18"/>
     </row>
@@ -4628,7 +4585,7 @@
       <c r="I47" s="12"/>
       <c r="J47" s="13">
         <f>0.13*G46*14817.6/5</f>
-        <v>10176.345328931937</v>
+        <v>7566.544976248997</v>
       </c>
       <c r="K47" s="12"/>
     </row>
@@ -4673,19 +4630,19 @@
         <v>1</v>
       </c>
       <c r="D50" s="14">
-        <f t="shared" ref="D50:F50" si="2">D10</f>
+        <f t="shared" ref="D50:F50" si="3">D10</f>
         <v>5</v>
       </c>
       <c r="E50" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.3907345321548306</v>
       </c>
       <c r="F50" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>0.12699380270242813</v>
       </c>
       <c r="G50" s="14">
-        <f t="shared" ref="G50:G65" si="3">PRODUCT(C50:F50)</f>
+        <f t="shared" ref="G50:G65" si="4">PRODUCT(C50:F50)</f>
         <v>2.1530113609639026</v>
       </c>
       <c r="H50" s="12"/>
@@ -4697,23 +4654,23 @@
       <c r="A51" s="10"/>
       <c r="B51" s="16"/>
       <c r="C51" s="12">
-        <f t="shared" ref="C51:F51" si="4">C11</f>
+        <f t="shared" ref="C51:F51" si="5">C11</f>
         <v>1</v>
       </c>
       <c r="D51" s="14">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="E51" s="14">
+        <f t="shared" si="5"/>
+        <v>3.3145382505333738</v>
+      </c>
+      <c r="F51" s="14">
+        <f t="shared" si="5"/>
+        <v>0.12699380270242813</v>
+      </c>
+      <c r="G51" s="14">
         <f t="shared" si="4"/>
-        <v>5</v>
-      </c>
-      <c r="E51" s="14">
-        <f t="shared" si="4"/>
-        <v>3.3145382505333738</v>
-      </c>
-      <c r="F51" s="14">
-        <f t="shared" si="4"/>
-        <v>0.12699380270242813</v>
-      </c>
-      <c r="G51" s="14">
-        <f t="shared" si="3"/>
         <v>2.1046290831894328</v>
       </c>
       <c r="H51" s="12"/>
@@ -4725,23 +4682,23 @@
       <c r="A52" s="10"/>
       <c r="B52" s="16"/>
       <c r="C52" s="12">
-        <f t="shared" ref="C52:F52" si="5">C12</f>
+        <f t="shared" ref="C52:F52" si="6">C12</f>
         <v>1</v>
       </c>
       <c r="D52" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>5</v>
       </c>
       <c r="E52" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>3.0219445291069795</v>
       </c>
       <c r="F52" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G52" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.571223876240704</v>
       </c>
       <c r="H52" s="12"/>
@@ -4753,23 +4710,23 @@
       <c r="A53" s="10"/>
       <c r="B53" s="16"/>
       <c r="C53" s="12">
-        <f t="shared" ref="C53:F53" si="6">C13</f>
+        <f t="shared" ref="C53:F53" si="7">C13</f>
         <v>1</v>
       </c>
       <c r="D53" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>5</v>
       </c>
       <c r="E53" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>2.9838463882962509</v>
       </c>
       <c r="F53" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.11033729553997765</v>
       </c>
       <c r="G53" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.6461477039566916</v>
       </c>
       <c r="H53" s="12"/>
@@ -4781,23 +4738,23 @@
       <c r="A54" s="10"/>
       <c r="B54" s="16"/>
       <c r="C54" s="12">
-        <f t="shared" ref="C54:F54" si="7">C14</f>
+        <f t="shared" ref="C54:F54" si="8">C14</f>
         <v>1</v>
       </c>
       <c r="D54" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>5</v>
       </c>
       <c r="E54" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>3.1621456872904599</v>
       </c>
       <c r="F54" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.11668698567509903</v>
       </c>
       <c r="G54" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.8449062425771903</v>
       </c>
       <c r="H54" s="12"/>
@@ -4809,23 +4766,23 @@
       <c r="A55" s="10"/>
       <c r="B55" s="16"/>
       <c r="C55" s="12">
-        <f t="shared" ref="C55:F55" si="8">C15</f>
+        <f t="shared" ref="C55:F55" si="9">C15</f>
         <v>1</v>
       </c>
       <c r="D55" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>5</v>
       </c>
       <c r="E55" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>3.0859494056690031</v>
       </c>
       <c r="F55" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.11668698567509903</v>
       </c>
       <c r="G55" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.8004506704668966</v>
       </c>
       <c r="H55" s="12"/>
@@ -4837,23 +4794,23 @@
       <c r="A56" s="10"/>
       <c r="B56" s="16"/>
       <c r="C56" s="12">
-        <f t="shared" ref="C56:F56" si="9">C16</f>
+        <f t="shared" ref="C56:F56" si="10">C16</f>
         <v>1</v>
       </c>
       <c r="D56" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>5</v>
       </c>
       <c r="E56" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.1366961292288935</v>
       </c>
       <c r="F56" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.11033729553997765</v>
       </c>
       <c r="G56" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.7304728391491617</v>
       </c>
       <c r="H56" s="12"/>
@@ -4865,23 +4822,23 @@
       <c r="A57" s="10"/>
       <c r="B57" s="16"/>
       <c r="C57" s="12">
-        <f t="shared" ref="C57:F57" si="10">C17</f>
+        <f t="shared" ref="C57:F57" si="11">C17</f>
         <v>1</v>
       </c>
       <c r="D57" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>5</v>
       </c>
       <c r="E57" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>3.1366961292288935</v>
       </c>
       <c r="F57" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G57" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.6308875968059711</v>
       </c>
       <c r="H57" s="12"/>
@@ -4893,23 +4850,23 @@
       <c r="A58" s="10"/>
       <c r="B58" s="16"/>
       <c r="C58" s="12">
-        <f t="shared" ref="C58:F58" si="11">C18</f>
+        <f t="shared" ref="C58:F58" si="12">C18</f>
         <v>1</v>
       </c>
       <c r="D58" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>5</v>
       </c>
       <c r="E58" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.1240475464797317</v>
       </c>
       <c r="F58" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G58" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.6243111176467186</v>
       </c>
       <c r="H58" s="12"/>
@@ -4921,23 +4878,23 @@
       <c r="A59" s="10"/>
       <c r="B59" s="16"/>
       <c r="C59" s="12">
-        <f t="shared" ref="C59:F59" si="12">C19</f>
+        <f t="shared" ref="C59:F59" si="13">C19</f>
         <v>1</v>
       </c>
       <c r="D59" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>5</v>
       </c>
       <c r="E59" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>3.2002438281011885</v>
       </c>
       <c r="F59" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>0.10398760540485627</v>
       </c>
       <c r="G59" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.6639284619795653</v>
       </c>
       <c r="H59" s="12"/>
@@ -4949,23 +4906,23 @@
       <c r="A60" s="10"/>
       <c r="B60" s="16"/>
       <c r="C60" s="12">
-        <f t="shared" ref="C60:F60" si="13">C20</f>
+        <f t="shared" ref="C60:F60" si="14">C20</f>
         <v>1</v>
       </c>
       <c r="D60" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>5</v>
       </c>
       <c r="E60" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>3.1240475464797317</v>
       </c>
       <c r="F60" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>7.8588844864370622E-2</v>
       </c>
       <c r="G60" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.2275764398960665</v>
       </c>
       <c r="H60" s="12"/>
@@ -4977,23 +4934,23 @@
       <c r="A61" s="10"/>
       <c r="B61" s="16"/>
       <c r="C61" s="12">
-        <f t="shared" ref="C61:F61" si="14">C21</f>
+        <f t="shared" ref="C61:F61" si="15">C21</f>
         <v>1</v>
       </c>
       <c r="D61" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3.047851264858275</v>
       </c>
       <c r="E61" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3.2002438281011885</v>
       </c>
       <c r="F61" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>6.5889464594127783E-2</v>
       </c>
       <c r="G61" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.64267708748628227</v>
       </c>
       <c r="H61" s="12"/>
@@ -5005,23 +4962,23 @@
       <c r="A62" s="10"/>
       <c r="B62" s="16"/>
       <c r="C62" s="12">
-        <f t="shared" ref="C62:F62" si="15">C22</f>
+        <f t="shared" ref="C62:F62" si="16">C22</f>
         <v>1</v>
       </c>
       <c r="D62" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>6</v>
       </c>
       <c r="E62" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>3.5557756781469063</v>
       </c>
       <c r="F62" s="14">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>0.15</v>
       </c>
       <c r="G62" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.2001981103322157</v>
       </c>
       <c r="H62" s="12"/>
@@ -5033,23 +4990,23 @@
       <c r="A63" s="10"/>
       <c r="B63" s="16"/>
       <c r="C63" s="12">
-        <f t="shared" ref="C63:F63" si="16">C23</f>
+        <f t="shared" ref="C63:F63" si="17">C23</f>
         <v>1</v>
       </c>
       <c r="D63" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.35558264756679875</v>
       </c>
       <c r="E63" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>3.8351112465711674</v>
       </c>
       <c r="F63" s="14">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.15</v>
       </c>
       <c r="G63" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.20455485161534726</v>
       </c>
       <c r="H63" s="12"/>
@@ -5061,23 +5018,23 @@
       <c r="A64" s="10"/>
       <c r="B64" s="16"/>
       <c r="C64" s="12">
-        <f t="shared" ref="C64:F64" si="17">C24</f>
+        <f t="shared" ref="C64:F64" si="18">C24</f>
         <v>1</v>
       </c>
       <c r="D64" s="14">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>5</v>
       </c>
       <c r="E64" s="14">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>4.4925556232855843</v>
       </c>
       <c r="F64" s="14">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.15</v>
       </c>
       <c r="G64" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.3694167174641878</v>
       </c>
       <c r="H64" s="12"/>
@@ -5089,24 +5046,24 @@
       <c r="A65" s="10"/>
       <c r="B65" s="16"/>
       <c r="C65" s="12">
-        <f t="shared" ref="C65:F65" si="18">C25</f>
-        <v>0</v>
+        <f t="shared" ref="C65:F65" si="19">C25</f>
+        <v>1</v>
       </c>
       <c r="D65" s="14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1</v>
       </c>
       <c r="E65" s="14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>5.6750000000000007</v>
       </c>
       <c r="F65" s="14">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.15</v>
       </c>
       <c r="G65" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f t="shared" si="4"/>
+        <v>0.85125000000000006</v>
       </c>
       <c r="H65" s="12"/>
       <c r="I65" s="12"/>
@@ -5124,7 +5081,7 @@
       <c r="F66" s="18"/>
       <c r="G66" s="19">
         <f>SUM(G50:G65)</f>
-        <v>26.414392159770337</v>
+        <v>27.265642159770337</v>
       </c>
       <c r="H66" s="20" t="s">
         <v>27</v>
@@ -5134,7 +5091,7 @@
       </c>
       <c r="J66" s="19">
         <f>G66*I66</f>
-        <v>316985.91311332391</v>
+        <v>327201.33873832395</v>
       </c>
       <c r="K66" s="18"/>
     </row>
@@ -5152,7 +5109,7 @@
       <c r="I67" s="12"/>
       <c r="J67" s="13">
         <f>0.13*G66*67891.51/15</f>
-        <v>15542.045735311067</v>
+        <v>16042.915350336069</v>
       </c>
       <c r="K67" s="12"/>
     </row>
@@ -5170,7 +5127,7 @@
       <c r="I68" s="12"/>
       <c r="J68" s="13">
         <f>0.13*G66*21432.6/15</f>
-        <v>4906.4522121636119</v>
+        <v>5064.5712186636119</v>
       </c>
       <c r="K68" s="12"/>
     </row>
@@ -5188,7 +5145,7 @@
       <c r="I69" s="12"/>
       <c r="J69" s="13">
         <f>0.13*G66*(27147.96+17146.08)/15</f>
-        <v>10140.001238471466</v>
+        <v>10466.780518571466</v>
       </c>
       <c r="K69" s="12"/>
     </row>
@@ -5206,7 +5163,7 @@
       <c r="I70" s="12"/>
       <c r="J70" s="13">
         <f>0.13*G66*775/15</f>
-        <v>177.41666733979076</v>
+        <v>183.13422983979078</v>
       </c>
       <c r="K70" s="12"/>
     </row>
@@ -5224,7 +5181,7 @@
       <c r="I71" s="12"/>
       <c r="J71" s="13">
         <f>0.13*G66*6923.4/15</f>
-        <v>1584.9374898842677</v>
+        <v>1636.0148733842677</v>
       </c>
       <c r="K71" s="12"/>
     </row>
@@ -5272,7 +5229,7 @@
         <f>B10</f>
         <v>-for road</v>
       </c>
-      <c r="C74" s="92">
+      <c r="C74" s="12">
         <v>16</v>
       </c>
       <c r="D74" s="14">
@@ -5306,27 +5263,27 @@
         <f>C74-N74</f>
         <v>0</v>
       </c>
-      <c r="P74" s="60"/>
+      <c r="P74" s="47"/>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="10"/>
       <c r="B75" s="16"/>
-      <c r="C75" s="92">
+      <c r="C75" s="12">
         <v>22</v>
       </c>
       <c r="D75" s="14">
         <v>2.9</v>
       </c>
       <c r="E75" s="14">
-        <f t="shared" ref="E75:E101" si="19">8*8/162</f>
+        <f t="shared" ref="E75:E101" si="20">8*8/162</f>
         <v>0.39506172839506171</v>
       </c>
       <c r="F75" s="12">
-        <f t="shared" ref="F75:F101" si="20">PRODUCT(C75:E75)</f>
+        <f t="shared" ref="F75:F101" si="21">PRODUCT(C75:E75)</f>
         <v>25.204938271604934</v>
       </c>
       <c r="G75" s="14">
-        <f t="shared" ref="G75:G101" si="21">F75/1000</f>
+        <f t="shared" ref="G75:G101" si="22">F75/1000</f>
         <v>2.5204938271604936E-2</v>
       </c>
       <c r="H75" s="12"/>
@@ -5338,34 +5295,34 @@
         <v>22.498285714285714</v>
       </c>
       <c r="N75" s="3">
-        <f t="shared" ref="N75:N101" si="22">TRUNC(M75,0)</f>
+        <f t="shared" ref="N75:N101" si="23">TRUNC(M75,0)</f>
         <v>22</v>
       </c>
       <c r="O75" s="3">
-        <f t="shared" ref="O75:O101" si="23">C75-N75</f>
+        <f t="shared" ref="O75:O101" si="24">C75-N75</f>
         <v>0</v>
       </c>
-      <c r="P75" s="60"/>
+      <c r="P75" s="47"/>
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="10"/>
       <c r="B76" s="16"/>
-      <c r="C76" s="92">
+      <c r="C76" s="12">
         <v>16</v>
       </c>
       <c r="D76" s="14">
         <v>4.12</v>
       </c>
       <c r="E76" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F76" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26.042469135802467</v>
       </c>
       <c r="G76" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.6042469135802465E-2</v>
       </c>
       <c r="H76" s="12"/>
@@ -5373,15 +5330,15 @@
       <c r="J76" s="13"/>
       <c r="K76" s="12"/>
       <c r="M76" s="3">
-        <f t="shared" ref="M76:M101" si="24">D77/(7/12/3.281)</f>
+        <f t="shared" ref="M76" si="25">D77/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N76" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O76" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5395,15 +5352,15 @@
         <v>2.94</v>
       </c>
       <c r="E77" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F77" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26.714074074074073</v>
       </c>
       <c r="G77" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.6714074074074074E-2</v>
       </c>
       <c r="H77" s="12"/>
@@ -5411,15 +5368,15 @@
       <c r="J77" s="13"/>
       <c r="K77" s="12"/>
       <c r="M77" s="3">
-        <f t="shared" ref="M77:M101" si="25">D76/(7/12/3.281)</f>
+        <f t="shared" ref="M77" si="26">D76/(7/12/3.281)</f>
         <v>23.173234285714287</v>
       </c>
       <c r="N77" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>23</v>
       </c>
       <c r="O77" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5433,15 +5390,15 @@
         <v>3.9</v>
       </c>
       <c r="E78" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F78" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.651851851851848</v>
       </c>
       <c r="G78" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4651851851851848E-2</v>
       </c>
       <c r="H78" s="12"/>
@@ -5449,15 +5406,15 @@
       <c r="J78" s="13"/>
       <c r="K78" s="12"/>
       <c r="M78" s="3">
-        <f t="shared" ref="M78:M101" si="26">D79/(7/12/3.281)</f>
+        <f t="shared" ref="M78" si="27">D79/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N78" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O78" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5471,15 +5428,15 @@
         <v>2.94</v>
       </c>
       <c r="E79" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F79" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.391111111111112</v>
       </c>
       <c r="G79" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4391111111111113E-2</v>
       </c>
       <c r="H79" s="12"/>
@@ -5487,15 +5444,15 @@
       <c r="J79" s="13"/>
       <c r="K79" s="12"/>
       <c r="M79" s="3">
-        <f t="shared" ref="M79:M101" si="27">D78/(7/12/3.281)</f>
+        <f t="shared" ref="M79" si="28">D78/(7/12/3.281)</f>
         <v>21.935828571428569</v>
       </c>
       <c r="N79" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>21</v>
       </c>
       <c r="O79" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5509,15 +5466,15 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="E80" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F80" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>30.222222222222221</v>
       </c>
       <c r="G80" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>3.022222222222222E-2</v>
       </c>
       <c r="H80" s="12"/>
@@ -5525,15 +5482,15 @@
       <c r="J80" s="13"/>
       <c r="K80" s="12"/>
       <c r="M80" s="3">
-        <f t="shared" ref="M80:M101" si="28">D81/(7/12/3.281)</f>
+        <f t="shared" ref="M80" si="29">D81/(7/12/3.281)</f>
         <v>15.186342857142858</v>
       </c>
       <c r="N80" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>15</v>
       </c>
       <c r="O80" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5547,15 +5504,15 @@
         <v>2.7</v>
       </c>
       <c r="E81" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F81" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>29.866666666666667</v>
       </c>
       <c r="G81" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.9866666666666666E-2</v>
       </c>
       <c r="H81" s="12"/>
@@ -5563,15 +5520,15 @@
       <c r="J81" s="13"/>
       <c r="K81" s="12"/>
       <c r="M81" s="3">
-        <f t="shared" ref="M81:M101" si="29">D80/(7/12/3.281)</f>
+        <f t="shared" ref="M81" si="30">D80/(7/12/3.281)</f>
         <v>28.685314285714284</v>
       </c>
       <c r="N81" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>28</v>
       </c>
       <c r="O81" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5585,15 +5542,15 @@
         <v>3.87</v>
       </c>
       <c r="E82" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F82" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.46222222222222</v>
       </c>
       <c r="G82" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4462222222222219E-2</v>
       </c>
       <c r="H82" s="12"/>
@@ -5601,15 +5558,15 @@
       <c r="J82" s="13"/>
       <c r="K82" s="12"/>
       <c r="M82" s="3">
-        <f t="shared" ref="M82:M101" si="30">D83/(7/12/3.281)</f>
+        <f t="shared" ref="M82" si="31">D83/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N82" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O82" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5623,15 +5580,15 @@
         <v>2.94</v>
       </c>
       <c r="E83" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F83" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.391111111111112</v>
       </c>
       <c r="G83" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4391111111111113E-2</v>
       </c>
       <c r="H83" s="12"/>
@@ -5639,15 +5596,15 @@
       <c r="J83" s="13"/>
       <c r="K83" s="12"/>
       <c r="M83" s="3">
-        <f t="shared" ref="M83:M101" si="31">D82/(7/12/3.281)</f>
+        <f t="shared" ref="M83" si="32">D82/(7/12/3.281)</f>
         <v>21.76709142857143</v>
       </c>
       <c r="N83" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>21</v>
       </c>
       <c r="O83" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5661,15 +5618,15 @@
         <v>4.0599999999999996</v>
       </c>
       <c r="E84" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F84" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25.663209876543206</v>
       </c>
       <c r="G84" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.5663209876543205E-2</v>
       </c>
       <c r="H84" s="12"/>
@@ -5677,15 +5634,15 @@
       <c r="J84" s="13"/>
       <c r="K84" s="12"/>
       <c r="M84" s="3">
-        <f t="shared" ref="M84:M101" si="32">D85/(7/12/3.281)</f>
+        <f t="shared" ref="M84" si="33">D85/(7/12/3.281)</f>
         <v>16.479994285714287</v>
       </c>
       <c r="N84" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O84" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5699,15 +5656,15 @@
         <v>2.93</v>
       </c>
       <c r="E85" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F85" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25.465679012345682</v>
       </c>
       <c r="G85" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.5465679012345682E-2</v>
       </c>
       <c r="H85" s="12"/>
@@ -5715,15 +5672,15 @@
       <c r="J85" s="13"/>
       <c r="K85" s="12"/>
       <c r="M85" s="3">
-        <f t="shared" ref="M85:M101" si="33">D84/(7/12/3.281)</f>
+        <f t="shared" ref="M85" si="34">D84/(7/12/3.281)</f>
         <v>22.835759999999997</v>
       </c>
       <c r="N85" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>22</v>
       </c>
       <c r="O85" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5737,15 +5694,15 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E86" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F86" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25.916049382716047</v>
       </c>
       <c r="G86" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.5916049382716046E-2</v>
       </c>
       <c r="H86" s="12"/>
@@ -5753,15 +5710,15 @@
       <c r="J86" s="13"/>
       <c r="K86" s="12"/>
       <c r="M86" s="3">
-        <f t="shared" ref="M86:M101" si="34">D87/(7/12/3.281)</f>
+        <f t="shared" ref="M86" si="35">D87/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N86" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O86" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5775,15 +5732,15 @@
         <v>2.94</v>
       </c>
       <c r="E87" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F87" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26.714074074074073</v>
       </c>
       <c r="G87" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.6714074074074074E-2</v>
       </c>
       <c r="H87" s="12"/>
@@ -5791,15 +5748,15 @@
       <c r="J87" s="13"/>
       <c r="K87" s="12"/>
       <c r="M87" s="3">
-        <f t="shared" ref="M87:M101" si="35">D86/(7/12/3.281)</f>
+        <f t="shared" ref="M87" si="36">D86/(7/12/3.281)</f>
         <v>23.060742857142856</v>
       </c>
       <c r="N87" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>23</v>
       </c>
       <c r="O87" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5813,15 +5770,15 @@
         <v>4.13</v>
       </c>
       <c r="E88" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F88" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.474074074074071</v>
       </c>
       <c r="G88" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4474074074074072E-2</v>
       </c>
       <c r="H88" s="12"/>
@@ -5829,15 +5786,15 @@
       <c r="J88" s="13"/>
       <c r="K88" s="12"/>
       <c r="M88" s="3">
-        <f t="shared" ref="M88:M101" si="36">D89/(7/12/3.281)</f>
+        <f t="shared" ref="M88" si="37">D89/(7/12/3.281)</f>
         <v>15.186342857142858</v>
       </c>
       <c r="N88" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>15</v>
       </c>
       <c r="O88" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5851,15 +5808,15 @@
         <v>2.7</v>
       </c>
       <c r="E89" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F89" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.533333333333331</v>
       </c>
       <c r="G89" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4533333333333331E-2</v>
       </c>
       <c r="H89" s="12"/>
@@ -5867,15 +5824,15 @@
       <c r="J89" s="13"/>
       <c r="K89" s="12"/>
       <c r="M89" s="3">
-        <f t="shared" ref="M89:M101" si="37">D88/(7/12/3.281)</f>
+        <f t="shared" ref="M89" si="38">D88/(7/12/3.281)</f>
         <v>23.229479999999999</v>
       </c>
       <c r="N89" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>23</v>
       </c>
       <c r="O89" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5889,15 +5846,15 @@
         <v>2.82</v>
       </c>
       <c r="E90" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F90" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>17.825185185185184</v>
       </c>
       <c r="G90" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1.7825185185185183E-2</v>
       </c>
       <c r="H90" s="12"/>
@@ -5905,15 +5862,15 @@
       <c r="J90" s="13"/>
       <c r="K90" s="12"/>
       <c r="M90" s="3">
-        <f t="shared" ref="M90:M101" si="38">D91/(7/12/3.281)</f>
+        <f t="shared" ref="M90" si="39">D91/(7/12/3.281)</f>
         <v>16.704977142857143</v>
       </c>
       <c r="N90" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O90" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5927,15 +5884,15 @@
         <v>2.97</v>
       </c>
       <c r="E91" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F91" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>17.600000000000001</v>
       </c>
       <c r="G91" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>1.7600000000000001E-2</v>
       </c>
       <c r="H91" s="12"/>
@@ -5943,15 +5900,15 @@
       <c r="J91" s="13"/>
       <c r="K91" s="12"/>
       <c r="M91" s="3">
-        <f t="shared" ref="M91:M101" si="39">D90/(7/12/3.281)</f>
+        <f t="shared" ref="M91" si="40">D90/(7/12/3.281)</f>
         <v>15.861291428571427</v>
       </c>
       <c r="N91" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>15</v>
       </c>
       <c r="O91" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -5965,15 +5922,15 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="E92" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F92" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25.916049382716047</v>
       </c>
       <c r="G92" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.5916049382716046E-2</v>
       </c>
       <c r="H92" s="12"/>
@@ -5981,15 +5938,15 @@
       <c r="J92" s="13"/>
       <c r="K92" s="12"/>
       <c r="M92" s="3">
-        <f t="shared" ref="M92:M101" si="40">D93/(7/12/3.281)</f>
+        <f t="shared" ref="M92" si="41">D93/(7/12/3.281)</f>
         <v>16.479994285714287</v>
       </c>
       <c r="N92" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O92" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6003,15 +5960,15 @@
         <v>2.93</v>
       </c>
       <c r="E93" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F93" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>26.623209876543207</v>
       </c>
       <c r="G93" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.6623209876543208E-2</v>
       </c>
       <c r="H93" s="12"/>
@@ -6019,15 +5976,15 @@
       <c r="J93" s="13"/>
       <c r="K93" s="12"/>
       <c r="M93" s="3">
-        <f t="shared" ref="M93:M101" si="41">D92/(7/12/3.281)</f>
+        <f t="shared" ref="M93" si="42">D92/(7/12/3.281)</f>
         <v>23.060742857142856</v>
       </c>
       <c r="N93" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>23</v>
       </c>
       <c r="O93" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6041,15 +5998,15 @@
         <v>3.55</v>
       </c>
       <c r="E94" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F94" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>22.439506172839504</v>
       </c>
       <c r="G94" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.2439506172839505E-2</v>
       </c>
       <c r="H94" s="12"/>
@@ -6057,15 +6014,15 @@
       <c r="J94" s="13"/>
       <c r="K94" s="12"/>
       <c r="M94" s="3">
-        <f t="shared" ref="M94:M101" si="42">D95/(7/12/3.281)</f>
+        <f t="shared" ref="M94" si="43">D95/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N94" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O94" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6079,15 +6036,15 @@
         <v>2.94</v>
       </c>
       <c r="E95" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F95" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>22.068148148148147</v>
       </c>
       <c r="G95" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.2068148148148146E-2</v>
       </c>
       <c r="H95" s="12"/>
@@ -6095,15 +6052,15 @@
       <c r="J95" s="13"/>
       <c r="K95" s="12"/>
       <c r="M95" s="3">
-        <f t="shared" ref="M95:M101" si="43">D94/(7/12/3.281)</f>
+        <f t="shared" ref="M95" si="44">D94/(7/12/3.281)</f>
         <v>19.967228571428571</v>
       </c>
       <c r="N95" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>19</v>
       </c>
       <c r="O95" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6117,15 +6074,15 @@
         <v>3.56</v>
       </c>
       <c r="E96" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F96" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>22.502716049382716</v>
       </c>
       <c r="G96" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.2502716049382716E-2</v>
       </c>
       <c r="H96" s="12"/>
@@ -6133,15 +6090,15 @@
       <c r="J96" s="13"/>
       <c r="K96" s="12"/>
       <c r="M96" s="3">
-        <f t="shared" ref="M96:M101" si="44">D97/(7/12/3.281)</f>
+        <f t="shared" ref="M96" si="45">D97/(7/12/3.281)</f>
         <v>16.536239999999999</v>
       </c>
       <c r="N96" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O96" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6155,15 +6112,15 @@
         <v>2.94</v>
       </c>
       <c r="E97" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F97" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>23.229629629629628</v>
       </c>
       <c r="G97" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.3229629629629628E-2</v>
       </c>
       <c r="H97" s="12"/>
@@ -6171,15 +6128,15 @@
       <c r="J97" s="13"/>
       <c r="K97" s="12"/>
       <c r="M97" s="3">
-        <f t="shared" ref="M97:M101" si="45">D96/(7/12/3.281)</f>
+        <f t="shared" ref="M97" si="46">D96/(7/12/3.281)</f>
         <v>20.023474285714286</v>
       </c>
       <c r="N97" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>20</v>
       </c>
       <c r="O97" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6193,15 +6150,15 @@
         <v>6.4</v>
       </c>
       <c r="E98" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F98" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>40.45432098765432</v>
       </c>
       <c r="G98" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>4.0454320987654321E-2</v>
       </c>
       <c r="H98" s="12"/>
@@ -6209,15 +6166,15 @@
       <c r="J98" s="13"/>
       <c r="K98" s="12"/>
       <c r="M98" s="3">
-        <f t="shared" ref="M98:M101" si="46">D99/(7/12/3.281)</f>
+        <f t="shared" ref="M98" si="47">D99/(7/12/3.281)</f>
         <v>16.479994285714287</v>
       </c>
       <c r="N98" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O98" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6231,15 +6188,15 @@
         <v>2.93</v>
       </c>
       <c r="E99" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F99" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>40.513580246913584</v>
       </c>
       <c r="G99" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>4.0513580246913587E-2</v>
       </c>
       <c r="H99" s="12"/>
@@ -6247,15 +6204,15 @@
       <c r="J99" s="13"/>
       <c r="K99" s="12"/>
       <c r="M99" s="3">
-        <f t="shared" ref="M99:M101" si="47">D98/(7/12/3.281)</f>
+        <f t="shared" ref="M99" si="48">D98/(7/12/3.281)</f>
         <v>35.997257142857144</v>
       </c>
       <c r="N99" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>35</v>
       </c>
       <c r="O99" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6269,15 +6226,15 @@
         <v>3.8</v>
       </c>
       <c r="E100" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F100" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.019753086419751</v>
       </c>
       <c r="G100" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4019753086419751E-2</v>
       </c>
       <c r="H100" s="12"/>
@@ -6285,15 +6242,15 @@
       <c r="J100" s="13"/>
       <c r="K100" s="12"/>
       <c r="M100" s="3">
-        <f t="shared" ref="M100:M101" si="48">D101/(7/12/3.281)</f>
+        <f t="shared" ref="M100" si="49">D101/(7/12/3.281)</f>
         <v>16.479994285714287</v>
       </c>
       <c r="N100" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>16</v>
       </c>
       <c r="O100" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6307,15 +6264,15 @@
         <v>2.93</v>
       </c>
       <c r="E101" s="14">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0.39506172839506171</v>
       </c>
       <c r="F101" s="12">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>24.308148148148149</v>
       </c>
       <c r="G101" s="14">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v>2.4308148148148148E-2</v>
       </c>
       <c r="H101" s="12"/>
@@ -6323,15 +6280,15 @@
       <c r="J101" s="13"/>
       <c r="K101" s="12"/>
       <c r="M101" s="3">
-        <f t="shared" ref="M101" si="49">D100/(7/12/3.281)</f>
+        <f t="shared" ref="M101" si="50">D100/(7/12/3.281)</f>
         <v>21.373371428571428</v>
       </c>
       <c r="N101" s="3">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v>21</v>
       </c>
       <c r="O101" s="3">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v>0</v>
       </c>
     </row>
@@ -6423,7 +6380,7 @@
       <c r="E106" s="18"/>
       <c r="F106" s="18"/>
       <c r="G106" s="20">
-        <f t="shared" ref="G106" si="50">PRODUCT(C106:F106)</f>
+        <f t="shared" ref="G106" si="51">PRODUCT(C106:F106)</f>
         <v>1</v>
       </c>
       <c r="H106" s="20" t="s">
@@ -6465,7 +6422,7 @@
       <c r="E108" s="18"/>
       <c r="F108" s="18"/>
       <c r="G108" s="20">
-        <f t="shared" ref="G108" si="51">PRODUCT(C108:F108)</f>
+        <f t="shared" ref="G108" si="52">PRODUCT(C108:F108)</f>
         <v>1</v>
       </c>
       <c r="H108" s="20" t="s">
@@ -6507,7 +6464,7 @@
       <c r="I110" s="13"/>
       <c r="J110" s="13">
         <f>SUM(J9:J108)</f>
-        <v>584751.77340097865</v>
+        <v>563256.49796061974</v>
       </c>
       <c r="K110" s="30"/>
     </row>
@@ -6516,11 +6473,11 @@
       <c r="B112" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="C112" s="47">
+      <c r="C112" s="72">
         <f>J110</f>
-        <v>584751.77340097865</v>
-      </c>
-      <c r="D112" s="48"/>
+        <v>563256.49796061974</v>
+      </c>
+      <c r="D112" s="73"/>
       <c r="E112" s="33">
         <v>100</v>
       </c>
@@ -6535,49 +6492,49 @@
       <c r="B113" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C113" s="51">
+      <c r="C113" s="76">
         <v>500000</v>
       </c>
-      <c r="D113" s="52"/>
+      <c r="D113" s="77"/>
       <c r="E113" s="33"/>
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B114" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="C114" s="51">
+      <c r="C114" s="76">
         <f>C113-C116-C117</f>
         <v>475000</v>
       </c>
-      <c r="D114" s="52"/>
+      <c r="D114" s="77"/>
       <c r="E114" s="33">
         <f>C114/C112*100</f>
-        <v>81.231049071873585</v>
+        <v>84.331028886454106</v>
       </c>
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B115" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C115" s="53">
+      <c r="C115" s="78">
         <f>C112-C114</f>
-        <v>109751.77340097865</v>
-      </c>
-      <c r="D115" s="53"/>
+        <v>88256.497960619745</v>
+      </c>
+      <c r="D115" s="78"/>
       <c r="E115" s="33">
         <f>100-E114</f>
-        <v>18.768950928126415</v>
+        <v>15.668971113545894</v>
       </c>
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B116" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="C116" s="47">
+      <c r="C116" s="72">
         <f>C113*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D116" s="48"/>
+      <c r="D116" s="73"/>
       <c r="E116" s="33">
         <v>3</v>
       </c>
@@ -6586,24 +6543,17 @@
       <c r="B117" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C117" s="47">
+      <c r="C117" s="72">
         <f>C113*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D117" s="48"/>
+      <c r="D117" s="73"/>
       <c r="E117" s="33">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C116:D116"/>
     <mergeCell ref="C117:D117"/>
     <mergeCell ref="A7:F7"/>
@@ -6612,6 +6562,13 @@
     <mergeCell ref="C113:D113"/>
     <mergeCell ref="C114:D114"/>
     <mergeCell ref="C115:D115"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>